<commit_message>
Fixing mixup between arginine and asparagine. Arginine was incorrectly labeled as asparagine
</commit_message>
<xml_diff>
--- a/data/raw/20260601_single_carbon_growth/Carbon_platemap_7.8.xlsx
+++ b/data/raw/20260601_single_carbon_growth/Carbon_platemap_7.8.xlsx
@@ -64,27 +64,7 @@
     <t xml:space="preserve">Medium/carbon source</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">M9MM with </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">arginine</t>
-    </r>
+    <t xml:space="preserve">M9MM with asparagine</t>
   </si>
   <si>
     <t xml:space="preserve">M9MM with cysteine</t>
@@ -112,7 +92,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -149,13 +129,6 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="4">
@@ -268,72 +241,68 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -589,6 +558,9 @@
   </sheetPr>
   <dimension ref="A1:N23"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24.34"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -979,12 +951,12 @@
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
       <c r="F10" s="13"/>
-      <c r="G10" s="14" t="s">
+      <c r="G10" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="13"/>
       <c r="K10" s="13" t="s">
         <v>16</v>
       </c>
@@ -995,18 +967,18 @@
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12"/>
       <c r="B11" s="2"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="15"/>
-      <c r="M11" s="15"/>
-      <c r="N11" s="15"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="14"/>
+      <c r="M11" s="14"/>
+      <c r="N11" s="14"/>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
@@ -1041,7 +1013,7 @@
       <c r="N13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="15" t="s">
         <v>17</v>
       </c>
       <c r="B14" s="2"/>
@@ -1365,12 +1337,12 @@
       <c r="D23" s="13"/>
       <c r="E23" s="13"/>
       <c r="F23" s="13"/>
-      <c r="G23" s="14" t="s">
+      <c r="G23" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="14"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
+      <c r="J23" s="13"/>
       <c r="K23" s="13" t="s">
         <v>20</v>
       </c>

</xml_diff>